<commit_message>
WIP: esquema battery swap en elmo_data.xlsx (320kW)
</commit_message>
<xml_diff>
--- a/data/Escenarios_Gx/320kW/elmo_data.xlsx
+++ b/data/Escenarios_Gx/320kW/elmo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_Gx\320kW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Escenarios_Gx\320kW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782BC8F8-F3CE-40CE-B3EA-BFA125998358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC12E43-E55E-4906-AF41-ACF12EAF6AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="4185" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="203">
   <si>
     <t>id</t>
   </si>
@@ -228,13 +228,7 @@
     <t>0.95</t>
   </si>
   <si>
-    <t>LH518B_2</t>
-  </si>
-  <si>
-    <t>LH518B_3</t>
-  </si>
-  <si>
-    <t>LH518B_4</t>
+    <t>swap_time</t>
   </si>
   <si>
     <t>LH518B</t>
@@ -531,6 +525,9 @@
     <t>USD</t>
   </si>
   <si>
+    <t>h</t>
+  </si>
+  <si>
     <t>station_1</t>
   </si>
   <si>
@@ -555,6 +552,15 @@
     <t>p_max_ssee</t>
   </si>
   <si>
+    <t>battery_cost</t>
+  </si>
+  <si>
+    <t>charge_time</t>
+  </si>
+  <si>
+    <t>Battery_swap</t>
+  </si>
+  <si>
     <t>type</t>
   </si>
   <si>
@@ -603,21 +609,27 @@
     <t>Bess</t>
   </si>
   <si>
-    <t>electric</t>
-  </si>
-  <si>
     <t>c_fixed</t>
   </si>
   <si>
     <t>c_bays</t>
   </si>
   <si>
+    <t>c_crane</t>
+  </si>
+  <si>
     <t>c_charger_space</t>
   </si>
   <si>
+    <t>c_battery_space</t>
+  </si>
+  <si>
     <t>max_bays</t>
   </si>
   <si>
+    <t>max_batteries_per_bay</t>
+  </si>
+  <si>
     <t>max_chargers_per_bay</t>
   </si>
   <si>
@@ -636,7 +648,7 @@
     <t>%</t>
   </si>
   <si>
-    <t>0.1</t>
+    <t>h_max</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1010,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1204,17 +1216,20 @@
     <xf numFmtId="3" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1522,38 +1537,37 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AC6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AE8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" style="23" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="23" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5703125" style="23" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.42578125" style="23" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" style="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" style="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.44140625" style="23" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7" style="23" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" style="23" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" style="24" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" style="23" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.6640625" style="24" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" style="23" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" style="23" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.5703125" style="24" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.109375" style="23" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.5546875" style="24" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18" style="24" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.85546875" style="24" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="20.85546875" style="24" customWidth="1"/>
-    <col min="24" max="24" width="18.42578125" style="24" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.140625" style="24" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.5703125" style="24" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="24" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="17" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="20.88671875" style="24" customWidth="1"/>
+    <col min="24" max="24" width="18.44140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.109375" style="24" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.5546875" style="24" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1641,8 +1655,14 @@
       <c r="AC1" s="27" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AD1" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE1" s="27" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="30" t="s">
         <v>3</v>
       </c>
@@ -1730,25 +1750,31 @@
       <c r="AC2" s="27" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="AD2" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="AE2" s="27" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31">
         <v>1</v>
       </c>
       <c r="B3" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="C3" t="s">
-        <v>160</v>
+      <c r="C3" s="38" t="s">
+        <v>158</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>52</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G3" s="9">
         <v>18</v>
@@ -1819,273 +1845,25 @@
       <c r="AC3" s="34" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A4" s="31">
-        <v>2</v>
-      </c>
-      <c r="B4" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="C4" t="s">
-        <v>160</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" s="9">
-        <v>18</v>
-      </c>
-      <c r="H4" s="22">
-        <v>0.84</v>
-      </c>
-      <c r="I4" s="9">
-        <v>20</v>
-      </c>
-      <c r="J4" s="9">
-        <v>20</v>
-      </c>
-      <c r="K4" s="9">
-        <v>52</v>
-      </c>
-      <c r="L4" s="9">
-        <v>540</v>
-      </c>
-      <c r="M4" s="22">
-        <v>6.26</v>
-      </c>
-      <c r="N4" s="35">
-        <v>-1</v>
-      </c>
-      <c r="O4" s="35">
-        <v>-1</v>
-      </c>
-      <c r="P4" s="35">
-        <v>-1</v>
-      </c>
-      <c r="Q4" s="35">
-        <v>-1</v>
-      </c>
-      <c r="R4" s="22">
-        <v>0.85</v>
-      </c>
-      <c r="S4" s="26">
-        <v>0.92</v>
-      </c>
-      <c r="T4" s="28">
-        <v>16.2</v>
-      </c>
-      <c r="U4" s="28">
-        <v>0.47</v>
-      </c>
-      <c r="V4" s="34">
-        <v>100</v>
-      </c>
-      <c r="W4" s="34">
-        <v>4</v>
-      </c>
-      <c r="X4" s="34">
-        <v>360</v>
-      </c>
-      <c r="Y4" s="34">
-        <v>4</v>
-      </c>
-      <c r="Z4" s="34">
-        <v>353</v>
-      </c>
-      <c r="AA4" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB4" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC4" s="34" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A5" s="31">
-        <v>3</v>
-      </c>
-      <c r="B5" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" t="s">
-        <v>160</v>
-      </c>
-      <c r="D5" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" s="9">
-        <v>18</v>
-      </c>
-      <c r="H5" s="22">
-        <v>0.84</v>
-      </c>
-      <c r="I5" s="9">
-        <v>20</v>
-      </c>
-      <c r="J5" s="9">
-        <v>20</v>
-      </c>
-      <c r="K5" s="9">
-        <v>52</v>
-      </c>
-      <c r="L5" s="9">
-        <v>540</v>
-      </c>
-      <c r="M5" s="22">
-        <v>6.26</v>
-      </c>
-      <c r="N5" s="35">
-        <v>-1</v>
-      </c>
-      <c r="O5" s="35">
-        <v>-1</v>
-      </c>
-      <c r="P5" s="35">
-        <v>-1</v>
-      </c>
-      <c r="Q5" s="35">
-        <v>-1</v>
-      </c>
-      <c r="R5" s="22">
-        <v>0.85</v>
-      </c>
-      <c r="S5" s="26">
-        <v>0.92</v>
-      </c>
-      <c r="T5" s="28">
-        <v>16.2</v>
-      </c>
-      <c r="U5" s="28">
-        <v>0.47</v>
-      </c>
-      <c r="V5" s="34">
-        <v>100</v>
-      </c>
-      <c r="W5" s="34">
-        <v>4</v>
-      </c>
-      <c r="X5" s="34">
-        <v>360</v>
-      </c>
-      <c r="Y5" s="34">
-        <v>4</v>
-      </c>
-      <c r="Z5" s="34">
-        <v>353</v>
-      </c>
-      <c r="AA5" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB5" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC5" s="34" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A6" s="31">
-        <v>4</v>
-      </c>
-      <c r="B6" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" t="s">
-        <v>160</v>
-      </c>
-      <c r="D6" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="F6" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="G6" s="9">
-        <v>18</v>
-      </c>
-      <c r="H6" s="22">
-        <v>0.84</v>
-      </c>
-      <c r="I6" s="9">
-        <v>20</v>
-      </c>
-      <c r="J6" s="9">
-        <v>20</v>
-      </c>
-      <c r="K6" s="9">
-        <v>52</v>
-      </c>
-      <c r="L6" s="9">
-        <v>540</v>
-      </c>
-      <c r="M6" s="22">
-        <v>6.26</v>
-      </c>
-      <c r="N6" s="35">
-        <v>-1</v>
-      </c>
-      <c r="O6" s="35">
-        <v>-1</v>
-      </c>
-      <c r="P6" s="35">
-        <v>-1</v>
-      </c>
-      <c r="Q6" s="35">
-        <v>-1</v>
-      </c>
-      <c r="R6" s="22">
-        <v>0.85</v>
-      </c>
-      <c r="S6" s="26">
-        <v>0.92</v>
-      </c>
-      <c r="T6" s="28">
-        <v>16.2</v>
-      </c>
-      <c r="U6" s="28">
-        <v>0.47</v>
-      </c>
-      <c r="V6" s="34">
-        <v>100</v>
-      </c>
-      <c r="W6" s="34">
-        <v>4</v>
-      </c>
-      <c r="X6" s="34">
-        <v>360</v>
-      </c>
-      <c r="Y6" s="34">
-        <v>4</v>
-      </c>
-      <c r="Z6" s="34">
-        <v>353</v>
-      </c>
-      <c r="AA6" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB6" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC6" s="34" t="s">
-        <v>61</v>
-      </c>
+      <c r="AD3" s="34">
+        <v>8.3000000000000004E-2</v>
+      </c>
+      <c r="AE3" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="Y7"/>
+      <c r="Z7"/>
+      <c r="AA7"/>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="Y8"/>
+      <c r="Z8"/>
+      <c r="AA8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -2095,91 +1873,106 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC93900-5A86-4519-AB89-460E8AC441EE}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>161</v>
+        <v>189</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>196</v>
+      </c>
+      <c r="J1" s="27" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="27" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>4</v>
+        <v>160</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E2" s="27" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>51</v>
+        <v>160</v>
       </c>
       <c r="G2" s="27" t="s">
         <v>51</v>
       </c>
       <c r="H2" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="J2" s="27" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="34">
-        <v>1</v>
-      </c>
-      <c r="B3" s="34" t="s">
-        <v>163</v>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="34">
+        <v>35722</v>
       </c>
       <c r="C3" s="34">
-        <v>35722</v>
+        <v>38221</v>
       </c>
       <c r="D3" s="34">
-        <v>38221</v>
+        <v>16752</v>
       </c>
       <c r="E3" s="34">
         <v>5733</v>
       </c>
       <c r="F3" s="34">
+        <v>4389</v>
+      </c>
+      <c r="G3" s="34">
         <v>2</v>
       </c>
-      <c r="G3" s="34">
-        <v>1</v>
-      </c>
       <c r="H3" s="34">
+        <v>2</v>
+      </c>
+      <c r="I3" s="34">
+        <v>2</v>
+      </c>
+      <c r="J3" s="34">
         <v>1500</v>
       </c>
     </row>
@@ -2191,30 +1984,36 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5C58D2-31A1-4CA6-99E5-3102447D41CF}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="C1" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="D1" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="E1" s="27" t="s">
         <v>166</v>
       </c>
-      <c r="E1" s="27" t="s">
+      <c r="F1" s="27" t="s">
         <v>167</v>
       </c>
-      <c r="F1" s="27" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="27" t="s">
+        <v>170</v>
+      </c>
+      <c r="H1" s="27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="27" t="s">
         <v>3</v>
       </c>
@@ -2222,7 +2021,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D2" s="27" t="s">
         <v>34</v>
@@ -2233,13 +2032,19 @@
       <c r="F2" s="27" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="H2" s="27" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C3" s="34">
         <v>42071</v>
@@ -2252,6 +2057,12 @@
       </c>
       <c r="F3" s="34">
         <v>5000</v>
+      </c>
+      <c r="G3" s="34">
+        <v>79000</v>
+      </c>
+      <c r="H3" s="34" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -2265,17 +2076,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H152"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="49" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.140625" style="69" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="49" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.109375" style="69" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
@@ -2301,7 +2112,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="51" t="s">
         <v>3</v>
       </c>
@@ -2327,12 +2138,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="52">
         <v>0</v>
       </c>
       <c r="B3" s="48" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C3" s="60" t="s">
         <v>6</v>
@@ -2353,12 +2164,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="53">
         <v>1</v>
       </c>
       <c r="B4" s="48" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C4" s="60" t="s">
         <v>6</v>
@@ -2379,12 +2190,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="53">
         <v>2</v>
       </c>
       <c r="B5" s="48" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C5" s="60" t="s">
         <v>6</v>
@@ -2405,12 +2216,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="52">
         <v>3</v>
       </c>
       <c r="B6" s="48" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C6" s="60" t="s">
         <v>6</v>
@@ -2431,12 +2242,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="53">
         <v>4</v>
       </c>
       <c r="B7" s="48" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C7" s="60" t="s">
         <v>6</v>
@@ -2457,12 +2268,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="53">
         <v>5</v>
       </c>
       <c r="B8" s="48" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C8" s="60" t="s">
         <v>6</v>
@@ -2483,12 +2294,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="52">
         <v>6</v>
       </c>
       <c r="B9" s="48" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C9" s="60" t="s">
         <v>6</v>
@@ -2509,12 +2320,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="53">
         <v>7</v>
       </c>
       <c r="B10" s="48" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C10" s="60" t="s">
         <v>6</v>
@@ -2535,12 +2346,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="53">
         <v>8</v>
       </c>
       <c r="B11" s="48" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C11" s="60" t="s">
         <v>6</v>
@@ -2561,12 +2372,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="52">
         <v>9</v>
       </c>
       <c r="B12" s="48" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C12" s="60" t="s">
         <v>6</v>
@@ -2587,12 +2398,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="53">
         <v>10</v>
       </c>
       <c r="B13" s="48" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C13" s="60" t="s">
         <v>6</v>
@@ -2613,12 +2424,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="53">
         <v>11</v>
       </c>
       <c r="B14" s="49" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C14" s="60" t="s">
         <v>6</v>
@@ -2639,12 +2450,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="53">
         <v>12</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C15" s="60" t="s">
         <v>6</v>
@@ -2665,12 +2476,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="52">
         <v>13</v>
       </c>
       <c r="B16" s="49" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C16" s="60" t="s">
         <v>6</v>
@@ -2691,12 +2502,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="53">
         <v>14</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C17" s="60" t="s">
         <v>6</v>
@@ -2717,12 +2528,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="53">
         <v>15</v>
       </c>
       <c r="B18" s="49" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C18" s="60" t="s">
         <v>6</v>
@@ -2743,12 +2554,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="52">
         <v>16</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C19" s="60" t="s">
         <v>6</v>
@@ -2769,12 +2580,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="53">
         <v>17</v>
       </c>
       <c r="B20" s="49" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C20" s="60" t="s">
         <v>6</v>
@@ -2795,12 +2606,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="53">
         <v>18</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C21" s="60" t="s">
         <v>6</v>
@@ -2821,12 +2632,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="52">
         <v>19</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C22" s="60" t="s">
         <v>6</v>
@@ -2847,12 +2658,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="53">
         <v>20</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C23" s="60" t="s">
         <v>6</v>
@@ -2873,12 +2684,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="53">
         <v>21</v>
       </c>
       <c r="B24" s="49" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C24" s="60" t="s">
         <v>6</v>
@@ -2899,12 +2710,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="53">
         <v>22</v>
       </c>
       <c r="B25" s="49" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C25" s="60" t="s">
         <v>6</v>
@@ -2925,12 +2736,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="52">
         <v>23</v>
       </c>
       <c r="B26" s="48" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C26" s="60" t="s">
         <v>13</v>
@@ -2951,12 +2762,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="53">
         <v>24</v>
       </c>
       <c r="B27" s="48" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C27" s="60" t="s">
         <v>13</v>
@@ -2977,12 +2788,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="52">
         <v>25</v>
       </c>
       <c r="B28" s="48" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C28" s="60" t="s">
         <v>13</v>
@@ -3003,12 +2814,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="53">
         <v>26</v>
       </c>
       <c r="B29" s="48" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C29" s="60" t="s">
         <v>13</v>
@@ -3029,12 +2840,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="53">
         <v>27</v>
       </c>
       <c r="B30" s="48" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C30" s="60" t="s">
         <v>13</v>
@@ -3055,12 +2866,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="52">
         <v>28</v>
       </c>
       <c r="B31" s="48" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C31" s="60" t="s">
         <v>13</v>
@@ -3081,12 +2892,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="53">
         <v>29</v>
       </c>
       <c r="B32" s="48" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C32" s="60" t="s">
         <v>13</v>
@@ -3107,12 +2918,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="53">
         <v>30</v>
       </c>
       <c r="B33" s="48" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C33" s="60" t="s">
         <v>13</v>
@@ -3133,12 +2944,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="52">
         <v>31</v>
       </c>
       <c r="B34" s="48" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C34" s="60" t="s">
         <v>13</v>
@@ -3159,12 +2970,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="53">
         <v>32</v>
       </c>
       <c r="B35" s="48" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C35" s="60" t="s">
         <v>13</v>
@@ -3185,12 +2996,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="53">
         <v>33</v>
       </c>
       <c r="B36" s="48" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C36" s="60" t="s">
         <v>13</v>
@@ -3211,12 +3022,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="52">
         <v>34</v>
       </c>
       <c r="B37" s="48" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C37" s="60" t="s">
         <v>13</v>
@@ -3237,12 +3048,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="53">
         <v>35</v>
       </c>
       <c r="B38" s="48" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C38" s="60" t="s">
         <v>13</v>
@@ -3263,12 +3074,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="53">
         <v>36</v>
       </c>
       <c r="B39" s="48" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C39" s="60" t="s">
         <v>13</v>
@@ -3289,12 +3100,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="53">
         <v>37</v>
       </c>
       <c r="B40" s="48" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C40" s="60" t="s">
         <v>13</v>
@@ -3315,12 +3126,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="52">
         <v>38</v>
       </c>
       <c r="B41" s="48" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C41" s="60" t="s">
         <v>13</v>
@@ -3341,12 +3152,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="53">
         <v>39</v>
       </c>
       <c r="B42" s="48" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C42" s="60" t="s">
         <v>13</v>
@@ -3367,12 +3178,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="53">
         <v>40</v>
       </c>
       <c r="B43" s="48" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C43" s="60" t="s">
         <v>13</v>
@@ -3393,12 +3204,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="53">
         <v>41</v>
       </c>
       <c r="B44" s="48" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C44" s="60" t="s">
         <v>13</v>
@@ -3419,12 +3230,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="53">
         <v>42</v>
       </c>
       <c r="B45" s="48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C45" s="60" t="s">
         <v>13</v>
@@ -3445,12 +3256,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="53">
         <v>43</v>
       </c>
       <c r="B46" s="48" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C46" s="60" t="s">
         <v>13</v>
@@ -3471,12 +3282,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="53">
         <v>44</v>
       </c>
       <c r="B47" s="48" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C47" s="60" t="s">
         <v>13</v>
@@ -3497,12 +3308,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="53">
         <v>45</v>
       </c>
       <c r="B48" s="48" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C48" s="60" t="s">
         <v>13</v>
@@ -3523,12 +3334,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="53">
         <v>46</v>
       </c>
       <c r="B49" s="48" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C49" s="60" t="s">
         <v>13</v>
@@ -3549,12 +3360,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="53">
         <v>47</v>
       </c>
       <c r="B50" s="48" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C50" s="60" t="s">
         <v>14</v>
@@ -3575,12 +3386,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="53">
         <v>48</v>
       </c>
       <c r="B51" s="48" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C51" s="60" t="s">
         <v>14</v>
@@ -3601,12 +3412,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="53">
         <v>49</v>
       </c>
       <c r="B52" s="48" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C52" s="60" t="s">
         <v>14</v>
@@ -3627,12 +3438,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="53">
         <v>50</v>
       </c>
       <c r="B53" s="48" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C53" s="60" t="s">
         <v>14</v>
@@ -3653,12 +3464,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="53">
         <v>51</v>
       </c>
       <c r="B54" s="48" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C54" s="60" t="s">
         <v>14</v>
@@ -3679,12 +3490,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="53">
         <v>52</v>
       </c>
       <c r="B55" s="48" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C55" s="60" t="s">
         <v>14</v>
@@ -3705,12 +3516,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="53">
         <v>53</v>
       </c>
       <c r="B56" s="48" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C56" s="60" t="s">
         <v>14</v>
@@ -3731,12 +3542,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="53">
         <v>54</v>
       </c>
       <c r="B57" s="48" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C57" s="60" t="s">
         <v>14</v>
@@ -3757,12 +3568,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="53">
         <v>55</v>
       </c>
       <c r="B58" s="48" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C58" s="60" t="s">
         <v>14</v>
@@ -3783,12 +3594,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="53">
         <v>56</v>
       </c>
       <c r="B59" s="48" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C59" s="60" t="s">
         <v>14</v>
@@ -3809,12 +3620,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="53">
         <v>57</v>
       </c>
       <c r="B60" s="48" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C60" s="60" t="s">
         <v>14</v>
@@ -3835,12 +3646,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="53">
         <v>58</v>
       </c>
       <c r="B61" s="48" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C61" s="60" t="s">
         <v>14</v>
@@ -3861,12 +3672,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="53">
         <v>59</v>
       </c>
       <c r="B62" s="48" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C62" s="60" t="s">
         <v>14</v>
@@ -3887,12 +3698,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="53">
         <v>60</v>
       </c>
       <c r="B63" s="48" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C63" s="60" t="s">
         <v>14</v>
@@ -3913,12 +3724,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="53">
         <v>61</v>
       </c>
       <c r="B64" s="48" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C64" s="60" t="s">
         <v>14</v>
@@ -3939,12 +3750,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="53">
         <v>62</v>
       </c>
       <c r="B65" s="48" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C65" s="60" t="s">
         <v>14</v>
@@ -3965,12 +3776,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="53">
         <v>63</v>
       </c>
       <c r="B66" s="48" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C66" s="60" t="s">
         <v>14</v>
@@ -3991,12 +3802,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="53">
         <v>64</v>
       </c>
       <c r="B67" s="48" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C67" s="60" t="s">
         <v>14</v>
@@ -4017,12 +3828,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="53">
         <v>65</v>
       </c>
       <c r="B68" s="48" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C68" s="60" t="s">
         <v>14</v>
@@ -4043,12 +3854,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="53">
         <v>66</v>
       </c>
       <c r="B69" s="48" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C69" s="60" t="s">
         <v>14</v>
@@ -4069,12 +3880,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="53">
         <v>67</v>
       </c>
       <c r="B70" s="48" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C70" s="60" t="s">
         <v>14</v>
@@ -4095,12 +3906,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="53">
         <v>68</v>
       </c>
       <c r="B71" s="48" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C71" s="60" t="s">
         <v>14</v>
@@ -4121,12 +3932,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="53">
         <v>69</v>
       </c>
       <c r="B72" s="48" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C72" s="60" t="s">
         <v>14</v>
@@ -4147,12 +3958,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="53">
         <v>70</v>
       </c>
       <c r="B73" s="48" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C73" s="60" t="s">
         <v>14</v>
@@ -4173,12 +3984,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="53">
         <v>71</v>
       </c>
       <c r="B74" s="48" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C74" s="60" t="s">
         <v>15</v>
@@ -4199,12 +4010,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="53">
         <v>72</v>
       </c>
       <c r="B75" s="48" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C75" s="60" t="s">
         <v>15</v>
@@ -4225,12 +4036,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="53">
         <v>73</v>
       </c>
       <c r="B76" s="48" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C76" s="60" t="s">
         <v>15</v>
@@ -4251,12 +4062,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="53">
         <v>74</v>
       </c>
       <c r="B77" s="48" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C77" s="60" t="s">
         <v>15</v>
@@ -4277,12 +4088,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="53">
         <v>75</v>
       </c>
       <c r="B78" s="48" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C78" s="60" t="s">
         <v>15</v>
@@ -4303,12 +4114,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="53">
         <v>76</v>
       </c>
       <c r="B79" s="48" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C79" s="60" t="s">
         <v>15</v>
@@ -4329,12 +4140,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="53">
         <v>77</v>
       </c>
       <c r="B80" s="48" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C80" s="60" t="s">
         <v>15</v>
@@ -4355,12 +4166,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="53">
         <v>78</v>
       </c>
       <c r="B81" s="48" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C81" s="60" t="s">
         <v>15</v>
@@ -4381,12 +4192,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="53">
         <v>79</v>
       </c>
       <c r="B82" s="48" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C82" s="60" t="s">
         <v>15</v>
@@ -4407,12 +4218,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="53">
         <v>80</v>
       </c>
       <c r="B83" s="48" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C83" s="60" t="s">
         <v>15</v>
@@ -4433,12 +4244,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="53">
         <v>81</v>
       </c>
       <c r="B84" s="48" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C84" s="60" t="s">
         <v>15</v>
@@ -4459,12 +4270,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="53">
         <v>82</v>
       </c>
       <c r="B85" s="48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C85" s="60" t="s">
         <v>15</v>
@@ -4485,12 +4296,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="53">
         <v>83</v>
       </c>
       <c r="B86" s="48" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C86" s="60" t="s">
         <v>15</v>
@@ -4511,12 +4322,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="53">
         <v>84</v>
       </c>
       <c r="B87" s="48" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C87" s="60" t="s">
         <v>15</v>
@@ -4537,12 +4348,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="53">
         <v>85</v>
       </c>
       <c r="B88" s="48" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C88" s="60" t="s">
         <v>15</v>
@@ -4563,12 +4374,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="53">
         <v>86</v>
       </c>
       <c r="B89" s="48" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C89" s="60" t="s">
         <v>15</v>
@@ -4589,12 +4400,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="53">
         <v>87</v>
       </c>
       <c r="B90" s="48" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C90" s="60" t="s">
         <v>15</v>
@@ -4615,12 +4426,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="53">
         <v>88</v>
       </c>
       <c r="B91" s="48" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C91" s="60" t="s">
         <v>15</v>
@@ -4641,12 +4452,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="53">
         <v>89</v>
       </c>
       <c r="B92" s="48" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C92" s="60" t="s">
         <v>15</v>
@@ -4667,12 +4478,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="53">
         <v>90</v>
       </c>
       <c r="B93" s="48" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C93" s="60" t="s">
         <v>15</v>
@@ -4693,12 +4504,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="53">
         <v>91</v>
       </c>
       <c r="B94" s="48" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C94" s="60" t="s">
         <v>15</v>
@@ -4719,12 +4530,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="53">
         <v>92</v>
       </c>
       <c r="B95" s="48" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C95" s="60" t="s">
         <v>15</v>
@@ -4745,12 +4556,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="53">
         <v>93</v>
       </c>
       <c r="B96" s="48" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C96" s="60" t="s">
         <v>15</v>
@@ -4771,16 +4582,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A97"/>
-      <c r="B97"/>
-      <c r="C97"/>
-      <c r="D97"/>
-      <c r="E97"/>
-      <c r="F97"/>
-      <c r="G97"/>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A97" s="53"/>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="54"/>
       <c r="B98" s="64"/>
       <c r="C98" s="61"/>
@@ -4788,7 +4593,7 @@
       <c r="G98" s="43"/>
       <c r="H98" s="44"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="55"/>
       <c r="B99" s="64"/>
       <c r="C99" s="62"/>
@@ -4796,7 +4601,7 @@
       <c r="G99" s="37"/>
       <c r="H99" s="8"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="56"/>
       <c r="B100" s="64"/>
       <c r="C100" s="62"/>
@@ -4804,7 +4609,7 @@
       <c r="G100" s="37"/>
       <c r="H100" s="8"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="57"/>
       <c r="B101" s="64"/>
       <c r="C101" s="62"/>
@@ -4812,7 +4617,7 @@
       <c r="G101" s="37"/>
       <c r="H101" s="8"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="57"/>
       <c r="B102" s="64"/>
       <c r="C102" s="62"/>
@@ -4820,7 +4625,7 @@
       <c r="G102" s="37"/>
       <c r="H102" s="8"/>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="57"/>
       <c r="B103" s="64"/>
       <c r="C103" s="62"/>
@@ -4828,7 +4633,7 @@
       <c r="G103" s="37"/>
       <c r="H103" s="8"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" s="55"/>
       <c r="B104" s="64"/>
       <c r="C104" s="62"/>
@@ -4836,7 +4641,7 @@
       <c r="G104" s="37"/>
       <c r="H104" s="8"/>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" s="56"/>
       <c r="B105" s="64"/>
       <c r="C105" s="62"/>
@@ -4844,7 +4649,7 @@
       <c r="G105" s="37"/>
       <c r="H105" s="8"/>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" s="57"/>
       <c r="B106" s="64"/>
       <c r="C106" s="62"/>
@@ -4852,7 +4657,7 @@
       <c r="G106" s="37"/>
       <c r="H106" s="8"/>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" s="57"/>
       <c r="B107" s="64"/>
       <c r="C107" s="62"/>
@@ -4860,7 +4665,7 @@
       <c r="G107" s="37"/>
       <c r="H107" s="8"/>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" s="57"/>
       <c r="B108" s="64"/>
       <c r="C108" s="62"/>
@@ -4868,7 +4673,7 @@
       <c r="G108" s="37"/>
       <c r="H108" s="8"/>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="55"/>
       <c r="B109" s="64"/>
       <c r="C109" s="62"/>
@@ -4876,7 +4681,7 @@
       <c r="G109" s="37"/>
       <c r="H109" s="8"/>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" s="56"/>
       <c r="B110" s="64"/>
       <c r="C110" s="62"/>
@@ -4884,7 +4689,7 @@
       <c r="G110" s="37"/>
       <c r="H110" s="8"/>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" s="57"/>
       <c r="B111" s="64"/>
       <c r="C111" s="62"/>
@@ -4892,7 +4697,7 @@
       <c r="G111" s="37"/>
       <c r="H111" s="8"/>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="57"/>
       <c r="B112" s="64"/>
       <c r="C112" s="62"/>
@@ -4900,7 +4705,7 @@
       <c r="G112" s="37"/>
       <c r="H112" s="8"/>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A113" s="57"/>
       <c r="B113" s="64"/>
       <c r="C113" s="62"/>
@@ -4908,7 +4713,7 @@
       <c r="G113" s="37"/>
       <c r="H113" s="8"/>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A114" s="55"/>
       <c r="B114" s="64"/>
       <c r="C114" s="62"/>
@@ -4916,7 +4721,7 @@
       <c r="G114" s="37"/>
       <c r="H114" s="8"/>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" s="56"/>
       <c r="B115" s="64"/>
       <c r="C115" s="62"/>
@@ -4924,7 +4729,7 @@
       <c r="G115" s="37"/>
       <c r="H115" s="8"/>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="57"/>
       <c r="B116" s="64"/>
       <c r="C116" s="62"/>
@@ -4932,7 +4737,7 @@
       <c r="G116" s="37"/>
       <c r="H116" s="8"/>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" s="57"/>
       <c r="B117" s="64"/>
       <c r="C117" s="62"/>
@@ -4940,7 +4745,7 @@
       <c r="G117" s="37"/>
       <c r="H117" s="8"/>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" s="57"/>
       <c r="B118" s="64"/>
       <c r="C118" s="62"/>
@@ -4948,7 +4753,7 @@
       <c r="G118" s="37"/>
       <c r="H118" s="8"/>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" s="55"/>
       <c r="B119" s="64"/>
       <c r="C119" s="62"/>
@@ -4956,7 +4761,7 @@
       <c r="G119" s="37"/>
       <c r="H119" s="8"/>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" s="56"/>
       <c r="B120" s="64"/>
       <c r="C120" s="62"/>
@@ -4964,7 +4769,7 @@
       <c r="G120" s="37"/>
       <c r="H120" s="8"/>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" s="57"/>
       <c r="B121" s="64"/>
       <c r="C121" s="62"/>
@@ -4972,7 +4777,7 @@
       <c r="G121" s="37"/>
       <c r="H121" s="8"/>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" s="57"/>
       <c r="B122" s="64"/>
       <c r="C122" s="62"/>
@@ -4980,7 +4785,7 @@
       <c r="G122" s="37"/>
       <c r="H122" s="8"/>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" s="57"/>
       <c r="B123" s="64"/>
       <c r="C123" s="62"/>
@@ -4988,7 +4793,7 @@
       <c r="G123" s="37"/>
       <c r="H123" s="8"/>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A124" s="55"/>
       <c r="B124" s="64"/>
       <c r="C124" s="62"/>
@@ -4996,7 +4801,7 @@
       <c r="G124" s="37"/>
       <c r="H124" s="8"/>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" s="56"/>
       <c r="B125" s="64"/>
       <c r="C125" s="62"/>
@@ -5004,7 +4809,7 @@
       <c r="G125" s="37"/>
       <c r="H125" s="8"/>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" s="57"/>
       <c r="B126" s="64"/>
       <c r="C126" s="62"/>
@@ -5012,7 +4817,7 @@
       <c r="G126" s="37"/>
       <c r="H126" s="8"/>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" s="57"/>
       <c r="B127" s="64"/>
       <c r="C127" s="62"/>
@@ -5020,7 +4825,7 @@
       <c r="G127" s="37"/>
       <c r="H127" s="8"/>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" s="57"/>
       <c r="B128" s="64"/>
       <c r="C128" s="62"/>
@@ -5028,7 +4833,7 @@
       <c r="G128" s="37"/>
       <c r="H128" s="8"/>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" s="55"/>
       <c r="B129" s="64"/>
       <c r="C129" s="62"/>
@@ -5036,7 +4841,7 @@
       <c r="G129" s="37"/>
       <c r="H129" s="8"/>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A130" s="56"/>
       <c r="B130" s="64"/>
       <c r="C130" s="62"/>
@@ -5044,7 +4849,7 @@
       <c r="G130" s="37"/>
       <c r="H130" s="8"/>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" s="57"/>
       <c r="B131" s="64"/>
       <c r="C131" s="62"/>
@@ -5052,7 +4857,7 @@
       <c r="G131" s="37"/>
       <c r="H131" s="8"/>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A132" s="57"/>
       <c r="B132" s="64"/>
       <c r="C132" s="62"/>
@@ -5060,7 +4865,7 @@
       <c r="G132" s="37"/>
       <c r="H132" s="8"/>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" s="57"/>
       <c r="B133" s="64"/>
       <c r="C133" s="62"/>
@@ -5068,7 +4873,7 @@
       <c r="G133" s="37"/>
       <c r="H133" s="8"/>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" s="55"/>
       <c r="B134" s="64"/>
       <c r="C134" s="62"/>
@@ -5076,7 +4881,7 @@
       <c r="G134" s="37"/>
       <c r="H134" s="8"/>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" s="56"/>
       <c r="B135" s="64"/>
       <c r="C135" s="62"/>
@@ -5084,7 +4889,7 @@
       <c r="G135" s="37"/>
       <c r="H135" s="8"/>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A136" s="57"/>
       <c r="B136" s="64"/>
       <c r="C136" s="62"/>
@@ -5092,7 +4897,7 @@
       <c r="G136" s="37"/>
       <c r="H136" s="8"/>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A137" s="57"/>
       <c r="B137" s="64"/>
       <c r="C137" s="62"/>
@@ -5100,7 +4905,7 @@
       <c r="G137" s="37"/>
       <c r="H137" s="8"/>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A138" s="57"/>
       <c r="B138" s="64"/>
       <c r="C138" s="62"/>
@@ -5108,7 +4913,7 @@
       <c r="G138" s="37"/>
       <c r="H138" s="8"/>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" s="55"/>
       <c r="B139" s="64"/>
       <c r="C139" s="62"/>
@@ -5116,7 +4921,7 @@
       <c r="G139" s="37"/>
       <c r="H139" s="8"/>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A140" s="56"/>
       <c r="B140" s="64"/>
       <c r="C140" s="62"/>
@@ -5124,7 +4929,7 @@
       <c r="G140" s="37"/>
       <c r="H140" s="8"/>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A141" s="57"/>
       <c r="B141" s="64"/>
       <c r="C141" s="62"/>
@@ -5132,7 +4937,7 @@
       <c r="G141" s="37"/>
       <c r="H141" s="8"/>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A142" s="57"/>
       <c r="B142" s="64"/>
       <c r="C142" s="62"/>
@@ -5140,7 +4945,7 @@
       <c r="G142" s="37"/>
       <c r="H142" s="8"/>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" s="57"/>
       <c r="B143" s="64"/>
       <c r="C143" s="62"/>
@@ -5148,7 +4953,7 @@
       <c r="G143" s="37"/>
       <c r="H143" s="8"/>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A144" s="55"/>
       <c r="B144" s="64"/>
       <c r="C144" s="62"/>
@@ -5156,7 +4961,7 @@
       <c r="G144" s="37"/>
       <c r="H144" s="8"/>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A145" s="56"/>
       <c r="B145" s="64"/>
       <c r="C145" s="62"/>
@@ -5164,7 +4969,7 @@
       <c r="G145" s="37"/>
       <c r="H145" s="8"/>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146" s="57"/>
       <c r="B146" s="64"/>
       <c r="C146" s="62"/>
@@ -5172,7 +4977,7 @@
       <c r="G146" s="37"/>
       <c r="H146" s="8"/>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147" s="57"/>
       <c r="B147" s="64"/>
       <c r="C147" s="62"/>
@@ -5180,7 +4985,7 @@
       <c r="G147" s="37"/>
       <c r="H147" s="8"/>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148" s="57"/>
       <c r="B148" s="64"/>
       <c r="C148" s="62"/>
@@ -5188,7 +4993,7 @@
       <c r="G148" s="37"/>
       <c r="H148" s="8"/>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A149" s="55"/>
       <c r="B149" s="64"/>
       <c r="C149" s="62"/>
@@ -5196,7 +5001,7 @@
       <c r="G149" s="37"/>
       <c r="H149" s="8"/>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A150" s="56"/>
       <c r="B150" s="64"/>
       <c r="C150" s="62"/>
@@ -5204,7 +5009,7 @@
       <c r="G150" s="37"/>
       <c r="H150" s="8"/>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A151" s="57"/>
       <c r="B151" s="64"/>
       <c r="C151" s="62"/>
@@ -5212,7 +5017,7 @@
       <c r="G151" s="37"/>
       <c r="H151" s="8"/>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A152" s="57"/>
       <c r="B152" s="64"/>
       <c r="C152" s="62"/>
@@ -5232,14 +5037,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5250,7 +5055,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -5261,7 +5066,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>0</v>
       </c>
@@ -5280,9 +5085,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C903B846-9155-4C37-ABE1-59FA4D45CD76}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5290,22 +5095,22 @@
         <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -5316,10 +5121,10 @@
         <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>34</v>
@@ -5328,15 +5133,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D3" s="3">
         <v>30.8</v>
@@ -5348,18 +5153,18 @@
         <v>500</v>
       </c>
       <c r="G3" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D4" s="3">
         <v>119</v>
@@ -5371,7 +5176,7 @@
         <v>500</v>
       </c>
       <c r="G4" s="3">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5381,13 +5186,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387AF5AC-D97C-4B95-B84B-AE3277E9ED2E}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5395,25 +5197,28 @@
         <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+      <c r="H1" s="70" t="s">
+        <v>186</v>
+      </c>
+      <c r="I1" s="71" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -5421,10 +5226,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>34</v>
@@ -5435,16 +5240,19 @@
       <c r="G2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="70" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" s="71" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C3" s="4">
         <v>18308</v>
@@ -5461,8 +5269,11 @@
       <c r="G3" s="3">
         <v>0</v>
       </c>
-      <c r="H3" s="3">
-        <v>1000</v>
+      <c r="H3" s="72">
+        <v>1000</v>
+      </c>
+      <c r="I3" s="75">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5471,34 +5282,35 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB361D3-2C0F-481F-8505-844CB2F9BDD0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE3F3123-4F4E-48AE-BFD8-F7DBC7028FBB}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="3.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D1" s="70" t="s">
-        <v>195</v>
-      </c>
-      <c r="E1" s="72" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+      <c r="E1" s="71" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>51</v>
       </c>
@@ -5506,30 +5318,30 @@
         <v>51</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D2" s="70" t="s">
-        <v>162</v>
-      </c>
-      <c r="E2" s="72" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="73">
+        <v>160</v>
+      </c>
+      <c r="E2" s="71" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="72">
         <v>1</v>
       </c>
       <c r="B3" s="34">
         <v>2.3532999999999998E-2</v>
       </c>
-      <c r="C3" s="74">
+      <c r="C3" s="73">
         <v>299000</v>
       </c>
-      <c r="D3" s="71">
+      <c r="D3" s="74">
         <v>0.8</v>
       </c>
-      <c r="E3" s="34" t="s">
-        <v>198</v>
+      <c r="E3" s="34">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>